<commit_message>
Block 4: Visualization Updates
</commit_message>
<xml_diff>
--- a/results/block3_results/cad-rads/Normal_1/patient_report_Normal_1.xlsx
+++ b/results/block3_results/cad-rads/Normal_1/patient_report_Normal_1.xlsx
@@ -799,10 +799,10 @@
         <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>115</v>
+        <v>460</v>
       </c>
       <c r="E2" t="n">
-        <v>89</v>
+        <v>356</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -842,10 +842,10 @@
         <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>405</v>
+        <v>1246</v>
       </c>
       <c r="E3" t="n">
-        <v>405</v>
+        <v>1246</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -885,10 +885,10 @@
         <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>333</v>
+        <v>925</v>
       </c>
       <c r="E4" t="n">
-        <v>333</v>
+        <v>925</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -971,10 +971,10 @@
         <v>0</v>
       </c>
       <c r="D6" t="n">
-        <v>72</v>
+        <v>363</v>
       </c>
       <c r="E6" t="n">
-        <v>43</v>
+        <v>160</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -1014,10 +1014,10 @@
         <v>0</v>
       </c>
       <c r="D7" t="n">
-        <v>215</v>
+        <v>776</v>
       </c>
       <c r="E7" t="n">
-        <v>215</v>
+        <v>776</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -1057,10 +1057,10 @@
         <v>0</v>
       </c>
       <c r="D8" t="n">
-        <v>110</v>
+        <v>206</v>
       </c>
       <c r="E8" t="n">
-        <v>95</v>
+        <v>191</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -1229,10 +1229,10 @@
         <v>0</v>
       </c>
       <c r="D12" t="n">
-        <v>158</v>
+        <v>268</v>
       </c>
       <c r="E12" t="n">
-        <v>158</v>
+        <v>268</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -1358,10 +1358,10 @@
         <v>0</v>
       </c>
       <c r="D15" t="n">
-        <v>606</v>
+        <v>804</v>
       </c>
       <c r="E15" t="n">
-        <v>535</v>
+        <v>729</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>

</xml_diff>